<commit_message>
MOD: Acertando testes, mudanças de relatórios e etc...
</commit_message>
<xml_diff>
--- a/tests/Caso de Teste_calcular_desconto.xlsx
+++ b/tests/Caso de Teste_calcular_desconto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20343"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENAI\Desktop\teste_desconto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENAI\Desktop\teste_desconto-main\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB27E4C9-4352-4FB4-9E5F-A6CC9A8B7718}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D40929B9-BDD1-453F-A31C-B0A79B2F002D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{B0A8FEDB-3CB4-46F9-981E-F499B3DD72A8}"/>
   </bookViews>
@@ -175,7 +175,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -184,11 +184,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="24"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Berlin Sans FB"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Berlin Sans FB"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -211,23 +216,119 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Berlin Sans FB"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Berlin Sans FB"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Berlin Sans FB"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Berlin Sans FB"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Berlin Sans FB"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Berlin Sans FB"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Berlin Sans FB"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -241,16 +342,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FDC16942-B2EA-4BE4-837F-6F65211ADB58}" name="Tabela2" displayName="Tabela2" ref="A3:E12" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FDC16942-B2EA-4BE4-837F-6F65211ADB58}" name="Tabela2" displayName="Tabela2" ref="A3:E12" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="A3:E12" xr:uid="{FE0308EA-E3D0-4768-9832-E2EEF7B68EAE}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{307D0158-9936-4E44-825F-723B4C63BC40}" name="Tipo de Teste"/>
-    <tableColumn id="2" xr3:uid="{9B6D87AB-33D9-4548-BC4D-5E4CE11A3653}" name="Função"/>
-    <tableColumn id="3" xr3:uid="{B345809D-5D2A-45CA-A057-4BAEAD1FD07E}" name="Descrição"/>
-    <tableColumn id="4" xr3:uid="{94997AD8-4221-4712-9A3F-AE464E099C9F}" name="Entrada"/>
-    <tableColumn id="5" xr3:uid="{7F63A259-84B9-4474-9D8A-9D912365FDB6}" name="Saída"/>
+    <tableColumn id="1" xr3:uid="{307D0158-9936-4E44-825F-723B4C63BC40}" name="Tipo de Teste" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{9B6D87AB-33D9-4548-BC4D-5E4CE11A3653}" name="Função" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{B345809D-5D2A-45CA-A057-4BAEAD1FD07E}" name="Descrição" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{94997AD8-4221-4712-9A3F-AE464E099C9F}" name="Entrada" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{7F63A259-84B9-4474-9D8A-9D912365FDB6}" name="Saída" dataDxfId="2"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleDark8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -264,7 +365,7 @@
     <tableColumn id="4" xr3:uid="{EF2DC11C-EEA3-4F07-8453-9A12766735B5}" name="Entrada"/>
     <tableColumn id="5" xr3:uid="{C08C73C7-C3E0-4847-A38B-AFAD89876EA8}" name="Saída"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleDark8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -576,314 +677,326 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="A7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="A9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="A10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="A11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="4" t="s">
         <v>31</v>
       </c>
     </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+    </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="A15" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>6</v>
-      </c>
-      <c r="B16" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="A16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>6</v>
-      </c>
-      <c r="B17" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="A17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="4" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="A18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B19" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="A19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="4" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="A20" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="4" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>6</v>
-      </c>
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="A21" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="4" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E22" s="2"/>
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="4"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="E23" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>